<commit_message>
fix: keep generate return aligned with scheduled output and warn on missing courses
Agent-Logs-Url: https://github.com/ArnavBallinCode/TimetableIIITDWD/sessions/bd454858-07dd-4930-9847-24a113a851a7

Co-authored-by: ArnavBallinCode <172006421+ArnavBallinCode@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Balanced_Timetable_latest.xlsx
+++ b/Balanced_Timetable_latest.xlsx
@@ -10246,10 +10246,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T34"/>
+  <dimension ref="A1:T38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="58" customWidth="1" min="1" max="1"/>
     <col width="43" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
@@ -10589,7 +10589,11 @@
       <c r="T8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>WARNING: Courses missing from generated timetable output</t>
+        </is>
+      </c>
       <c r="B9" s="4" t="n"/>
       <c r="C9" s="4" t="n"/>
       <c r="D9" s="4" t="n"/>
@@ -10611,7 +10615,11 @@
       <c r="T9" s="4" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DS308: combined-course constraints prevented placement</t>
+        </is>
+      </c>
       <c r="B10" s="4" t="n"/>
       <c r="C10" s="4" t="n"/>
       <c r="D10" s="4" t="n"/>
@@ -10633,11 +10641,7 @@
       <c r="T10" s="4" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>DSAI-IV Second Half</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
       <c r="B11" s="4" t="n"/>
       <c r="C11" s="4" t="n"/>
       <c r="D11" s="4" t="n"/>
@@ -10659,214 +10663,186 @@
       <c r="T11" s="4" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>07:30-09:00</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>09:00-10:00</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>10:00-10:30</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>10:30-10:45</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>10:45-11:00</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>11:00-12:00</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>12:00-12:15</t>
-        </is>
-      </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>12:15-12:30</t>
-        </is>
-      </c>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>12:30-12:45</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="inlineStr">
-        <is>
-          <t>12:45-13:15</t>
-        </is>
-      </c>
-      <c r="L12" s="3" t="inlineStr">
-        <is>
-          <t>13:15-14:00</t>
-        </is>
-      </c>
-      <c r="M12" s="3" t="inlineStr">
-        <is>
-          <t>14:00-14:30</t>
-        </is>
-      </c>
-      <c r="N12" s="3" t="inlineStr">
-        <is>
-          <t>14:30-15:30</t>
-        </is>
-      </c>
-      <c r="O12" s="3" t="inlineStr">
-        <is>
-          <t>15:30-15:40</t>
-        </is>
-      </c>
-      <c r="P12" s="3" t="inlineStr">
-        <is>
-          <t>15:40-16:00</t>
-        </is>
-      </c>
-      <c r="Q12" s="3" t="inlineStr">
-        <is>
-          <t>16:00-16:30</t>
-        </is>
-      </c>
-      <c r="R12" s="3" t="inlineStr">
-        <is>
-          <t>16:30-17:10</t>
-        </is>
-      </c>
-      <c r="S12" s="3" t="inlineStr">
-        <is>
-          <t>17:10-17:30</t>
-        </is>
-      </c>
-      <c r="T12" s="3" t="inlineStr">
-        <is>
-          <t>17:30-18:30</t>
-        </is>
-      </c>
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" s="4" t="n"/>
+      <c r="C12" s="4" t="n"/>
+      <c r="D12" s="4" t="n"/>
+      <c r="E12" s="4" t="n"/>
+      <c r="F12" s="4" t="n"/>
+      <c r="G12" s="4" t="n"/>
+      <c r="H12" s="4" t="n"/>
+      <c r="I12" s="4" t="n"/>
+      <c r="J12" s="4" t="n"/>
+      <c r="K12" s="4" t="n"/>
+      <c r="L12" s="4" t="n"/>
+      <c r="M12" s="4" t="n"/>
+      <c r="N12" s="4" t="n"/>
+      <c r="O12" s="4" t="n"/>
+      <c r="P12" s="4" t="n"/>
+      <c r="Q12" s="4" t="n"/>
+      <c r="R12" s="4" t="n"/>
+      <c r="S12" s="4" t="n"/>
+      <c r="T12" s="4" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Monday</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr"/>
-      <c r="C13" s="11" t="inlineStr">
-        <is>
-          <t>Elective2</t>
-        </is>
-      </c>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="4" t="inlineStr"/>
-      <c r="F13" s="29" t="inlineStr">
-        <is>
-          <t>DA263T (C403)</t>
-        </is>
-      </c>
-      <c r="G13" s="29" t="n"/>
-      <c r="H13" s="4" t="inlineStr"/>
-      <c r="I13" s="4" t="inlineStr"/>
-      <c r="J13" s="4" t="inlineStr"/>
-      <c r="K13" s="4" t="inlineStr"/>
-      <c r="L13" s="4" t="inlineStr"/>
-      <c r="M13" s="28" t="inlineStr">
-        <is>
-          <t>DA265 (C405)</t>
-        </is>
-      </c>
-      <c r="N13" s="28" t="n"/>
-      <c r="O13" s="4" t="inlineStr"/>
-      <c r="P13" s="4" t="inlineStr"/>
-      <c r="Q13" s="4" t="inlineStr"/>
-      <c r="R13" s="4" t="inlineStr"/>
-      <c r="S13" s="4" t="inlineStr"/>
-      <c r="T13" s="4" t="inlineStr"/>
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>DSAI-IV Second Half</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n"/>
+      <c r="C13" s="4" t="n"/>
+      <c r="D13" s="4" t="n"/>
+      <c r="E13" s="4" t="n"/>
+      <c r="F13" s="4" t="n"/>
+      <c r="G13" s="4" t="n"/>
+      <c r="H13" s="4" t="n"/>
+      <c r="I13" s="4" t="n"/>
+      <c r="J13" s="4" t="n"/>
+      <c r="K13" s="4" t="n"/>
+      <c r="L13" s="4" t="n"/>
+      <c r="M13" s="4" t="n"/>
+      <c r="N13" s="4" t="n"/>
+      <c r="O13" s="4" t="n"/>
+      <c r="P13" s="4" t="n"/>
+      <c r="Q13" s="4" t="n"/>
+      <c r="R13" s="4" t="n"/>
+      <c r="S13" s="4" t="n"/>
+      <c r="T13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Tuesday</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr"/>
-      <c r="C14" s="11" t="inlineStr">
-        <is>
-          <t>Elective2</t>
-        </is>
-      </c>
-      <c r="D14" s="11" t="n"/>
-      <c r="E14" s="4" t="inlineStr"/>
-      <c r="F14" s="27" t="inlineStr">
-        <is>
-          <t>DA264 (C404)</t>
-        </is>
-      </c>
-      <c r="G14" s="27" t="n"/>
-      <c r="H14" s="27" t="n"/>
-      <c r="I14" s="28" t="inlineStr">
-        <is>
-          <t>DA265T (C405)</t>
-        </is>
-      </c>
-      <c r="J14" s="28" t="n"/>
-      <c r="K14" s="28" t="n"/>
-      <c r="L14" s="4" t="inlineStr"/>
-      <c r="M14" s="4" t="inlineStr"/>
-      <c r="N14" s="4" t="inlineStr"/>
-      <c r="O14" s="4" t="inlineStr"/>
-      <c r="P14" s="4" t="inlineStr"/>
-      <c r="Q14" s="4" t="inlineStr"/>
-      <c r="R14" s="4" t="inlineStr"/>
-      <c r="S14" s="4" t="inlineStr"/>
-      <c r="T14" s="4" t="inlineStr"/>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>07:30-09:00</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>09:00-10:00</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>10:00-10:30</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>10:30-10:45</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>10:45-11:00</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>11:00-12:00</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>12:00-12:15</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>12:15-12:30</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>12:30-12:45</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>12:45-13:15</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>13:15-14:00</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>14:00-14:30</t>
+        </is>
+      </c>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>14:30-15:30</t>
+        </is>
+      </c>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t>15:30-15:40</t>
+        </is>
+      </c>
+      <c r="P14" s="3" t="inlineStr">
+        <is>
+          <t>15:40-16:00</t>
+        </is>
+      </c>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>16:00-16:30</t>
+        </is>
+      </c>
+      <c r="R14" s="3" t="inlineStr">
+        <is>
+          <t>16:30-17:10</t>
+        </is>
+      </c>
+      <c r="S14" s="3" t="inlineStr">
+        <is>
+          <t>17:10-17:30</t>
+        </is>
+      </c>
+      <c r="T14" s="3" t="inlineStr">
+        <is>
+          <t>17:30-18:30</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Monday</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr"/>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Elective2T</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr"/>
+          <t>Elective2</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="n"/>
       <c r="E15" s="4" t="inlineStr"/>
-      <c r="F15" s="27" t="inlineStr">
-        <is>
-          <t>DA264 (C404)</t>
-        </is>
-      </c>
-      <c r="G15" s="27" t="n"/>
-      <c r="H15" s="27" t="n"/>
+      <c r="F15" s="29" t="inlineStr">
+        <is>
+          <t>DA263T (C403)</t>
+        </is>
+      </c>
+      <c r="G15" s="29" t="n"/>
+      <c r="H15" s="4" t="inlineStr"/>
       <c r="I15" s="4" t="inlineStr"/>
       <c r="J15" s="4" t="inlineStr"/>
       <c r="K15" s="4" t="inlineStr"/>
       <c r="L15" s="4" t="inlineStr"/>
-      <c r="M15" s="25" t="inlineStr">
-        <is>
-          <t>HS261 (C403)</t>
-        </is>
-      </c>
-      <c r="N15" s="25" t="n"/>
+      <c r="M15" s="28" t="inlineStr">
+        <is>
+          <t>DA265 (C405)</t>
+        </is>
+      </c>
+      <c r="N15" s="28" t="n"/>
       <c r="O15" s="4" t="inlineStr"/>
       <c r="P15" s="4" t="inlineStr"/>
       <c r="Q15" s="4" t="inlineStr"/>
@@ -10877,34 +10853,34 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Thursday</t>
+          <t>Tuesday</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr"/>
-      <c r="C16" s="29" t="inlineStr">
-        <is>
-          <t>DA263 (C403)</t>
-        </is>
-      </c>
-      <c r="D16" s="29" t="n"/>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Elective2</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="n"/>
       <c r="E16" s="4" t="inlineStr"/>
       <c r="F16" s="27" t="inlineStr">
         <is>
-          <t>DA264 (Lab-L406)</t>
+          <t>DA264 (C404)</t>
         </is>
       </c>
       <c r="G16" s="27" t="n"/>
       <c r="H16" s="27" t="n"/>
-      <c r="I16" s="27" t="n"/>
-      <c r="J16" s="27" t="n"/>
-      <c r="K16" s="4" t="inlineStr"/>
+      <c r="I16" s="28" t="inlineStr">
+        <is>
+          <t>DA265T (C405)</t>
+        </is>
+      </c>
+      <c r="J16" s="28" t="n"/>
+      <c r="K16" s="28" t="n"/>
       <c r="L16" s="4" t="inlineStr"/>
-      <c r="M16" s="25" t="inlineStr">
-        <is>
-          <t>HS261 (C403)</t>
-        </is>
-      </c>
-      <c r="N16" s="25" t="n"/>
+      <c r="M16" s="4" t="inlineStr"/>
+      <c r="N16" s="4" t="inlineStr"/>
       <c r="O16" s="4" t="inlineStr"/>
       <c r="P16" s="4" t="inlineStr"/>
       <c r="Q16" s="4" t="inlineStr"/>
@@ -10915,30 +10891,34 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Friday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr"/>
-      <c r="C17" s="28" t="inlineStr">
-        <is>
-          <t>DA265 (C405)</t>
-        </is>
-      </c>
-      <c r="D17" s="28" t="n"/>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Elective2T</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr"/>
       <c r="E17" s="4" t="inlineStr"/>
-      <c r="F17" s="29" t="inlineStr">
-        <is>
-          <t>DA263 (C403)</t>
-        </is>
-      </c>
-      <c r="G17" s="29" t="n"/>
-      <c r="H17" s="29" t="n"/>
+      <c r="F17" s="27" t="inlineStr">
+        <is>
+          <t>DA264 (C404)</t>
+        </is>
+      </c>
+      <c r="G17" s="27" t="n"/>
+      <c r="H17" s="27" t="n"/>
       <c r="I17" s="4" t="inlineStr"/>
       <c r="J17" s="4" t="inlineStr"/>
       <c r="K17" s="4" t="inlineStr"/>
       <c r="L17" s="4" t="inlineStr"/>
-      <c r="M17" s="4" t="inlineStr"/>
-      <c r="N17" s="4" t="inlineStr"/>
+      <c r="M17" s="25" t="inlineStr">
+        <is>
+          <t>HS261 (C403)</t>
+        </is>
+      </c>
+      <c r="N17" s="25" t="n"/>
       <c r="O17" s="4" t="inlineStr"/>
       <c r="P17" s="4" t="inlineStr"/>
       <c r="Q17" s="4" t="inlineStr"/>
@@ -10947,51 +10927,83 @@
       <c r="T17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
-      <c r="B18" s="4" t="n"/>
-      <c r="C18" s="4" t="n"/>
-      <c r="D18" s="4" t="n"/>
-      <c r="E18" s="4" t="n"/>
-      <c r="F18" s="4" t="n"/>
-      <c r="G18" s="4" t="n"/>
-      <c r="H18" s="4" t="n"/>
-      <c r="I18" s="4" t="n"/>
-      <c r="J18" s="4" t="n"/>
-      <c r="K18" s="4" t="n"/>
-      <c r="L18" s="4" t="n"/>
-      <c r="M18" s="4" t="n"/>
-      <c r="N18" s="4" t="n"/>
-      <c r="O18" s="4" t="n"/>
-      <c r="P18" s="4" t="n"/>
-      <c r="Q18" s="4" t="n"/>
-      <c r="R18" s="4" t="n"/>
-      <c r="S18" s="4" t="n"/>
-      <c r="T18" s="4" t="n"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr"/>
+      <c r="C18" s="29" t="inlineStr">
+        <is>
+          <t>DA263 (C403)</t>
+        </is>
+      </c>
+      <c r="D18" s="29" t="n"/>
+      <c r="E18" s="4" t="inlineStr"/>
+      <c r="F18" s="27" t="inlineStr">
+        <is>
+          <t>DA264 (Lab-L406)</t>
+        </is>
+      </c>
+      <c r="G18" s="27" t="n"/>
+      <c r="H18" s="27" t="n"/>
+      <c r="I18" s="27" t="n"/>
+      <c r="J18" s="27" t="n"/>
+      <c r="K18" s="4" t="inlineStr"/>
+      <c r="L18" s="4" t="inlineStr"/>
+      <c r="M18" s="25" t="inlineStr">
+        <is>
+          <t>HS261 (C403)</t>
+        </is>
+      </c>
+      <c r="N18" s="25" t="n"/>
+      <c r="O18" s="4" t="inlineStr"/>
+      <c r="P18" s="4" t="inlineStr"/>
+      <c r="Q18" s="4" t="inlineStr"/>
+      <c r="R18" s="4" t="inlineStr"/>
+      <c r="S18" s="4" t="inlineStr"/>
+      <c r="T18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
-      <c r="B19" s="4" t="n"/>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="4" t="n"/>
-      <c r="E19" s="4" t="n"/>
-      <c r="F19" s="4" t="n"/>
-      <c r="G19" s="4" t="n"/>
-      <c r="H19" s="4" t="n"/>
-      <c r="I19" s="4" t="n"/>
-      <c r="J19" s="4" t="n"/>
-      <c r="K19" s="4" t="n"/>
-      <c r="L19" s="4" t="n"/>
-      <c r="M19" s="4" t="n"/>
-      <c r="N19" s="4" t="n"/>
-      <c r="O19" s="4" t="n"/>
-      <c r="P19" s="4" t="n"/>
-      <c r="Q19" s="4" t="n"/>
-      <c r="R19" s="4" t="n"/>
-      <c r="S19" s="4" t="n"/>
-      <c r="T19" s="4" t="n"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr"/>
+      <c r="C19" s="28" t="inlineStr">
+        <is>
+          <t>DA265 (C405)</t>
+        </is>
+      </c>
+      <c r="D19" s="28" t="n"/>
+      <c r="E19" s="4" t="inlineStr"/>
+      <c r="F19" s="29" t="inlineStr">
+        <is>
+          <t>DA263 (C403)</t>
+        </is>
+      </c>
+      <c r="G19" s="29" t="n"/>
+      <c r="H19" s="29" t="n"/>
+      <c r="I19" s="4" t="inlineStr"/>
+      <c r="J19" s="4" t="inlineStr"/>
+      <c r="K19" s="4" t="inlineStr"/>
+      <c r="L19" s="4" t="inlineStr"/>
+      <c r="M19" s="4" t="inlineStr"/>
+      <c r="N19" s="4" t="inlineStr"/>
+      <c r="O19" s="4" t="inlineStr"/>
+      <c r="P19" s="4" t="inlineStr"/>
+      <c r="Q19" s="4" t="inlineStr"/>
+      <c r="R19" s="4" t="inlineStr"/>
+      <c r="S19" s="4" t="inlineStr"/>
+      <c r="T19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>WARNING: Courses missing from generated timetable output</t>
+        </is>
+      </c>
       <c r="B20" s="4" t="n"/>
       <c r="C20" s="4" t="n"/>
       <c r="D20" s="4" t="n"/>
@@ -11013,9 +11025,9 @@
       <c r="T20" s="4" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="inlineStr">
-        <is>
-          <t>Legend - DSAI IV</t>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>DS308: combined-course constraints prevented placement</t>
         </is>
       </c>
       <c r="B21" s="4" t="n"/>
@@ -11039,46 +11051,14 @@
       <c r="T21" s="4" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="14" t="inlineStr">
-        <is>
-          <t>Course Code</t>
-        </is>
-      </c>
-      <c r="B22" s="15" t="inlineStr">
-        <is>
-          <t>Course Title</t>
-        </is>
-      </c>
-      <c r="C22" s="15" t="inlineStr">
-        <is>
-          <t>L-T-P-S-C</t>
-        </is>
-      </c>
-      <c r="D22" s="15" t="inlineStr">
-        <is>
-          <t>Faculty</t>
-        </is>
-      </c>
-      <c r="E22" s="15" t="inlineStr">
-        <is>
-          <t>Semester Half</t>
-        </is>
-      </c>
-      <c r="F22" s="16" t="inlineStr">
-        <is>
-          <t>Elective</t>
-        </is>
-      </c>
-      <c r="G22" s="16" t="inlineStr">
-        <is>
-          <t>Elective Basket</t>
-        </is>
-      </c>
-      <c r="H22" s="16" t="inlineStr">
-        <is>
-          <t>Elective Room</t>
-        </is>
-      </c>
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" s="4" t="n"/>
+      <c r="C22" s="4" t="n"/>
+      <c r="D22" s="4" t="n"/>
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="n"/>
+      <c r="G22" s="4" t="n"/>
+      <c r="H22" s="4" t="n"/>
       <c r="I22" s="4" t="n"/>
       <c r="J22" s="4" t="n"/>
       <c r="K22" s="4" t="n"/>
@@ -11093,42 +11073,14 @@
       <c r="T22" s="4" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="inlineStr">
-        <is>
-          <t>DA263</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Big Data Analytics</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>3-1-0-0-4</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>Dr. Animesh Chaturvedi</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>Full Sem</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr"/>
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" s="4" t="n"/>
+      <c r="C23" s="4" t="n"/>
+      <c r="D23" s="4" t="n"/>
+      <c r="E23" s="4" t="n"/>
+      <c r="F23" s="4" t="n"/>
+      <c r="G23" s="4" t="n"/>
+      <c r="H23" s="4" t="n"/>
       <c r="I23" s="4" t="n"/>
       <c r="J23" s="4" t="n"/>
       <c r="K23" s="4" t="n"/>
@@ -11143,42 +11095,14 @@
       <c r="T23" s="4" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="17" t="inlineStr">
-        <is>
-          <t>DA264</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Database Management and Warehousing</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>3-0-2-0-4</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>Dr. Utkarsh Mahadeo Khaire</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>Full Sem</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr"/>
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" s="4" t="n"/>
+      <c r="C24" s="4" t="n"/>
+      <c r="D24" s="4" t="n"/>
+      <c r="E24" s="4" t="n"/>
+      <c r="F24" s="4" t="n"/>
+      <c r="G24" s="4" t="n"/>
+      <c r="H24" s="4" t="n"/>
       <c r="I24" s="4" t="n"/>
       <c r="J24" s="4" t="n"/>
       <c r="K24" s="4" t="n"/>
@@ -11193,42 +11117,18 @@
       <c r="T24" s="4" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="17" t="inlineStr">
-        <is>
-          <t>DA265</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>Deep Learning</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>3-1-0-0-4</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>Dr. Shirshendu Layek</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>Full Sem</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr"/>
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>Legend - DSAI IV</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n"/>
+      <c r="C25" s="4" t="n"/>
+      <c r="D25" s="4" t="n"/>
+      <c r="E25" s="4" t="n"/>
+      <c r="F25" s="4" t="n"/>
+      <c r="G25" s="4" t="n"/>
+      <c r="H25" s="4" t="n"/>
       <c r="I25" s="4" t="n"/>
       <c r="J25" s="4" t="n"/>
       <c r="K25" s="4" t="n"/>
@@ -11243,42 +11143,46 @@
       <c r="T25" s="4" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="17" t="inlineStr">
-        <is>
-          <t>DS308</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>Data Security and Privacy</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>3-1-0-4-4</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>Dr. Girish Revadigar</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>Full Sem</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr"/>
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>Course Code</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>Course Title</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="inlineStr">
+        <is>
+          <t>L-T-P-S-C</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="inlineStr">
+        <is>
+          <t>Faculty</t>
+        </is>
+      </c>
+      <c r="E26" s="15" t="inlineStr">
+        <is>
+          <t>Semester Half</t>
+        </is>
+      </c>
+      <c r="F26" s="16" t="inlineStr">
+        <is>
+          <t>Elective</t>
+        </is>
+      </c>
+      <c r="G26" s="16" t="inlineStr">
+        <is>
+          <t>Elective Basket</t>
+        </is>
+      </c>
+      <c r="H26" s="16" t="inlineStr">
+        <is>
+          <t>Elective Room</t>
+        </is>
+      </c>
       <c r="I26" s="4" t="n"/>
       <c r="J26" s="4" t="n"/>
       <c r="K26" s="4" t="n"/>
@@ -11295,22 +11199,22 @@
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
         <is>
-          <t>HS261</t>
+          <t>DA263</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Ethics and Values / Environmental Studies</t>
+          <t>Big Data Analytics</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>3-0-0-0-3</t>
+          <t>3-1-0-0-4</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Dr. Aswath Babu H</t>
+          <t>Dr. Animesh Chaturvedi</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -11345,44 +11249,40 @@
     <row r="28">
       <c r="A28" s="17" t="inlineStr">
         <is>
-          <t>EC255</t>
+          <t>DA264</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Embedded Intelligent Sensing Systems</t>
+          <t>Database Management and Warehousing</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>2-0-2-4-2</t>
+          <t>3-0-2-0-4</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Dr. Sibasankar Padhy</t>
+          <t>Dr. Utkarsh Mahadeo Khaire</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>First Half</t>
+          <t>Full Sem</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H28" s="3" t="inlineStr">
-        <is>
-          <t>C301</t>
-        </is>
-      </c>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr"/>
       <c r="I28" s="4" t="n"/>
       <c r="J28" s="4" t="n"/>
       <c r="K28" s="4" t="n"/>
@@ -11399,44 +11299,40 @@
     <row r="29">
       <c r="A29" s="17" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>DA265</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Edge AI Systems Design</t>
+          <t>Deep Learning</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>3-1-0-0-2</t>
+          <t>3-1-0-0-4</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Dr. Deepak K T</t>
+          <t>Dr. Shirshendu Layek</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>First Half</t>
+          <t>Full Sem</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr">
-        <is>
-          <t>C102</t>
-        </is>
-      </c>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr"/>
       <c r="I29" s="4" t="n"/>
       <c r="J29" s="4" t="n"/>
       <c r="K29" s="4" t="n"/>
@@ -11453,44 +11349,40 @@
     <row r="30">
       <c r="A30" s="17" t="inlineStr">
         <is>
-          <t>CS252</t>
+          <t>DS308</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Digital Forensic</t>
+          <t>Data Security and Privacy</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>3-1-0-0-2</t>
+          <t>3-1-0-4-4</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Dr. Abdul Wahid</t>
+          <t>Dr. Girish Revadigar</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Second Half</t>
+          <t>Full Sem</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>C401</t>
-        </is>
-      </c>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr"/>
       <c r="I30" s="4" t="n"/>
       <c r="J30" s="4" t="n"/>
       <c r="K30" s="4" t="n"/>
@@ -11507,44 +11399,40 @@
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>CS261</t>
+          <t>HS261</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Operating System</t>
+          <t>Ethics and Values / Environmental Studies</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>3-1-0-0-2</t>
+          <t>3-0-0-0-3</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Dr. Siddharth R</t>
+          <t>Dr. Aswath Babu H</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Second Half</t>
+          <t>Full Sem</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr">
-        <is>
-          <t>C003</t>
-        </is>
-      </c>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr"/>
       <c r="I31" s="4" t="n"/>
       <c r="J31" s="4" t="n"/>
       <c r="K31" s="4" t="n"/>
@@ -11561,27 +11449,27 @@
     <row r="32">
       <c r="A32" s="17" t="inlineStr">
         <is>
-          <t>EC257</t>
+          <t>EC255</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Causal Inference</t>
+          <t>Embedded Intelligent Sensing Systems</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>3-1-0-0-2</t>
+          <t>2-0-2-4-2</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Dr. Chinmayananda A</t>
+          <t>Dr. Sibasankar Padhy</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Second Half</t>
+          <t>First Half</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
@@ -11591,12 +11479,12 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>C302</t>
+          <t>C301</t>
         </is>
       </c>
       <c r="I32" s="4" t="n"/>
@@ -11615,12 +11503,12 @@
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>CS253</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Time Series Forecasting and Applications</t>
+          <t>Edge AI Systems Design</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -11630,12 +11518,12 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Dr. Nataraj</t>
+          <t>Dr. Deepak K T</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Second Half</t>
+          <t>First Half</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
@@ -11645,12 +11533,12 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>C303</t>
+          <t>C102</t>
         </is>
       </c>
       <c r="I33" s="4" t="n"/>
@@ -11667,14 +11555,46 @@
       <c r="T33" s="4" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr"/>
-      <c r="B34" s="4" t="n"/>
-      <c r="C34" s="4" t="n"/>
-      <c r="D34" s="4" t="n"/>
-      <c r="E34" s="4" t="n"/>
-      <c r="F34" s="4" t="n"/>
-      <c r="G34" s="4" t="n"/>
-      <c r="H34" s="4" t="n"/>
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>CS252</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Digital Forensic</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>3-1-0-0-2</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Abdul Wahid</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Second Half</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>C401</t>
+        </is>
+      </c>
       <c r="I34" s="4" t="n"/>
       <c r="J34" s="4" t="n"/>
       <c r="K34" s="4" t="n"/>
@@ -11688,32 +11608,216 @@
       <c r="S34" s="4" t="n"/>
       <c r="T34" s="4" t="n"/>
     </row>
+    <row r="35">
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>CS261</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Operating System</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>3-1-0-0-2</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Siddharth R</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Second Half</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>C003</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="n"/>
+      <c r="J35" s="4" t="n"/>
+      <c r="K35" s="4" t="n"/>
+      <c r="L35" s="4" t="n"/>
+      <c r="M35" s="4" t="n"/>
+      <c r="N35" s="4" t="n"/>
+      <c r="O35" s="4" t="n"/>
+      <c r="P35" s="4" t="n"/>
+      <c r="Q35" s="4" t="n"/>
+      <c r="R35" s="4" t="n"/>
+      <c r="S35" s="4" t="n"/>
+      <c r="T35" s="4" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="17" t="inlineStr">
+        <is>
+          <t>EC257</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Causal Inference</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>3-1-0-0-2</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Chinmayananda A</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Second Half</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>C302</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="n"/>
+      <c r="J36" s="4" t="n"/>
+      <c r="K36" s="4" t="n"/>
+      <c r="L36" s="4" t="n"/>
+      <c r="M36" s="4" t="n"/>
+      <c r="N36" s="4" t="n"/>
+      <c r="O36" s="4" t="n"/>
+      <c r="P36" s="4" t="n"/>
+      <c r="Q36" s="4" t="n"/>
+      <c r="R36" s="4" t="n"/>
+      <c r="S36" s="4" t="n"/>
+      <c r="T36" s="4" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="17" t="inlineStr">
+        <is>
+          <t>CS253</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Time Series Forecasting and Applications</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>3-1-0-0-2</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Nataraj</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Second Half</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>C303</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="n"/>
+      <c r="J37" s="4" t="n"/>
+      <c r="K37" s="4" t="n"/>
+      <c r="L37" s="4" t="n"/>
+      <c r="M37" s="4" t="n"/>
+      <c r="N37" s="4" t="n"/>
+      <c r="O37" s="4" t="n"/>
+      <c r="P37" s="4" t="n"/>
+      <c r="Q37" s="4" t="n"/>
+      <c r="R37" s="4" t="n"/>
+      <c r="S37" s="4" t="n"/>
+      <c r="T37" s="4" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+      <c r="B38" s="4" t="n"/>
+      <c r="C38" s="4" t="n"/>
+      <c r="D38" s="4" t="n"/>
+      <c r="E38" s="4" t="n"/>
+      <c r="F38" s="4" t="n"/>
+      <c r="G38" s="4" t="n"/>
+      <c r="H38" s="4" t="n"/>
+      <c r="I38" s="4" t="n"/>
+      <c r="J38" s="4" t="n"/>
+      <c r="K38" s="4" t="n"/>
+      <c r="L38" s="4" t="n"/>
+      <c r="M38" s="4" t="n"/>
+      <c r="N38" s="4" t="n"/>
+      <c r="O38" s="4" t="n"/>
+      <c r="P38" s="4" t="n"/>
+      <c r="Q38" s="4" t="n"/>
+      <c r="R38" s="4" t="n"/>
+      <c r="S38" s="4" t="n"/>
+      <c r="T38" s="4" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="I16:K16"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="F5:H5"/>
+    <mergeCell ref="C15:D15"/>
     <mergeCell ref="O4:Q4"/>
-    <mergeCell ref="F16:J16"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="F8:H8"/>
-    <mergeCell ref="C14:D14"/>
     <mergeCell ref="M5:N5"/>
     <mergeCell ref="F17:H17"/>
     <mergeCell ref="F6:J6"/>
+    <mergeCell ref="C18:D18"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="C16:D16"/>
-    <mergeCell ref="I14:K14"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="F18:J18"/>
     <mergeCell ref="M15:N15"/>
-    <mergeCell ref="F14:H14"/>
     <mergeCell ref="M6:N6"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="F16:H16"/>
     <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="F19:H19"/>
+    <mergeCell ref="C19:D19"/>
     <mergeCell ref="F7:H7"/>
-    <mergeCell ref="F15:H15"/>
     <mergeCell ref="M4:N4"/>
     <mergeCell ref="F4:J4"/>
   </mergeCells>

</xml_diff>

<commit_message>
chore: revert generated timetable workbook artifact
Agent-Logs-Url: https://github.com/ArnavBallinCode/TimetableIIITDWD/sessions/bd454858-07dd-4930-9847-24a113a851a7

Co-authored-by: ArnavBallinCode <172006421+ArnavBallinCode@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Balanced_Timetable_latest.xlsx
+++ b/Balanced_Timetable_latest.xlsx
@@ -10246,10 +10246,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T38"/>
+  <dimension ref="A1:T34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
     <col width="43" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
@@ -10589,11 +10589,7 @@
       <c r="T8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>WARNING: Courses missing from generated timetable output</t>
-        </is>
-      </c>
+      <c r="A9" t="inlineStr"/>
       <c r="B9" s="4" t="n"/>
       <c r="C9" s="4" t="n"/>
       <c r="D9" s="4" t="n"/>
@@ -10615,11 +10611,7 @@
       <c r="T9" s="4" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>DS308: combined-course constraints prevented placement</t>
-        </is>
-      </c>
+      <c r="A10" t="inlineStr"/>
       <c r="B10" s="4" t="n"/>
       <c r="C10" s="4" t="n"/>
       <c r="D10" s="4" t="n"/>
@@ -10641,7 +10633,11 @@
       <c r="T10" s="4" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>DSAI-IV Second Half</t>
+        </is>
+      </c>
       <c r="B11" s="4" t="n"/>
       <c r="C11" s="4" t="n"/>
       <c r="D11" s="4" t="n"/>
@@ -10663,186 +10659,214 @@
       <c r="T11" s="4" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="4" t="n"/>
-      <c r="E12" s="4" t="n"/>
-      <c r="F12" s="4" t="n"/>
-      <c r="G12" s="4" t="n"/>
-      <c r="H12" s="4" t="n"/>
-      <c r="I12" s="4" t="n"/>
-      <c r="J12" s="4" t="n"/>
-      <c r="K12" s="4" t="n"/>
-      <c r="L12" s="4" t="n"/>
-      <c r="M12" s="4" t="n"/>
-      <c r="N12" s="4" t="n"/>
-      <c r="O12" s="4" t="n"/>
-      <c r="P12" s="4" t="n"/>
-      <c r="Q12" s="4" t="n"/>
-      <c r="R12" s="4" t="n"/>
-      <c r="S12" s="4" t="n"/>
-      <c r="T12" s="4" t="n"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>07:30-09:00</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>09:00-10:00</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>10:00-10:30</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>10:30-10:45</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>10:45-11:00</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>11:00-12:00</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>12:00-12:15</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>12:15-12:30</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>12:30-12:45</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>12:45-13:15</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>13:15-14:00</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>14:00-14:30</t>
+        </is>
+      </c>
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>14:30-15:30</t>
+        </is>
+      </c>
+      <c r="O12" s="3" t="inlineStr">
+        <is>
+          <t>15:30-15:40</t>
+        </is>
+      </c>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>15:40-16:00</t>
+        </is>
+      </c>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>16:00-16:30</t>
+        </is>
+      </c>
+      <c r="R12" s="3" t="inlineStr">
+        <is>
+          <t>16:30-17:10</t>
+        </is>
+      </c>
+      <c r="S12" s="3" t="inlineStr">
+        <is>
+          <t>17:10-17:30</t>
+        </is>
+      </c>
+      <c r="T12" s="3" t="inlineStr">
+        <is>
+          <t>17:30-18:30</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>DSAI-IV Second Half</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
-      <c r="D13" s="4" t="n"/>
-      <c r="E13" s="4" t="n"/>
-      <c r="F13" s="4" t="n"/>
-      <c r="G13" s="4" t="n"/>
-      <c r="H13" s="4" t="n"/>
-      <c r="I13" s="4" t="n"/>
-      <c r="J13" s="4" t="n"/>
-      <c r="K13" s="4" t="n"/>
-      <c r="L13" s="4" t="n"/>
-      <c r="M13" s="4" t="n"/>
-      <c r="N13" s="4" t="n"/>
-      <c r="O13" s="4" t="n"/>
-      <c r="P13" s="4" t="n"/>
-      <c r="Q13" s="4" t="n"/>
-      <c r="R13" s="4" t="n"/>
-      <c r="S13" s="4" t="n"/>
-      <c r="T13" s="4" t="n"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr"/>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Elective2</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="4" t="inlineStr"/>
+      <c r="F13" s="29" t="inlineStr">
+        <is>
+          <t>DA263T (C403)</t>
+        </is>
+      </c>
+      <c r="G13" s="29" t="n"/>
+      <c r="H13" s="4" t="inlineStr"/>
+      <c r="I13" s="4" t="inlineStr"/>
+      <c r="J13" s="4" t="inlineStr"/>
+      <c r="K13" s="4" t="inlineStr"/>
+      <c r="L13" s="4" t="inlineStr"/>
+      <c r="M13" s="28" t="inlineStr">
+        <is>
+          <t>DA265 (C405)</t>
+        </is>
+      </c>
+      <c r="N13" s="28" t="n"/>
+      <c r="O13" s="4" t="inlineStr"/>
+      <c r="P13" s="4" t="inlineStr"/>
+      <c r="Q13" s="4" t="inlineStr"/>
+      <c r="R13" s="4" t="inlineStr"/>
+      <c r="S13" s="4" t="inlineStr"/>
+      <c r="T13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>07:30-09:00</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>09:00-10:00</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>10:00-10:30</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>10:30-10:45</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>10:45-11:00</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>11:00-12:00</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
-        <is>
-          <t>12:00-12:15</t>
-        </is>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>12:15-12:30</t>
-        </is>
-      </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>12:30-12:45</t>
-        </is>
-      </c>
-      <c r="K14" s="3" t="inlineStr">
-        <is>
-          <t>12:45-13:15</t>
-        </is>
-      </c>
-      <c r="L14" s="3" t="inlineStr">
-        <is>
-          <t>13:15-14:00</t>
-        </is>
-      </c>
-      <c r="M14" s="3" t="inlineStr">
-        <is>
-          <t>14:00-14:30</t>
-        </is>
-      </c>
-      <c r="N14" s="3" t="inlineStr">
-        <is>
-          <t>14:30-15:30</t>
-        </is>
-      </c>
-      <c r="O14" s="3" t="inlineStr">
-        <is>
-          <t>15:30-15:40</t>
-        </is>
-      </c>
-      <c r="P14" s="3" t="inlineStr">
-        <is>
-          <t>15:40-16:00</t>
-        </is>
-      </c>
-      <c r="Q14" s="3" t="inlineStr">
-        <is>
-          <t>16:00-16:30</t>
-        </is>
-      </c>
-      <c r="R14" s="3" t="inlineStr">
-        <is>
-          <t>16:30-17:10</t>
-        </is>
-      </c>
-      <c r="S14" s="3" t="inlineStr">
-        <is>
-          <t>17:10-17:30</t>
-        </is>
-      </c>
-      <c r="T14" s="3" t="inlineStr">
-        <is>
-          <t>17:30-18:30</t>
-        </is>
-      </c>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr"/>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Elective2</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="4" t="inlineStr"/>
+      <c r="F14" s="27" t="inlineStr">
+        <is>
+          <t>DA264 (C404)</t>
+        </is>
+      </c>
+      <c r="G14" s="27" t="n"/>
+      <c r="H14" s="27" t="n"/>
+      <c r="I14" s="28" t="inlineStr">
+        <is>
+          <t>DA265T (C405)</t>
+        </is>
+      </c>
+      <c r="J14" s="28" t="n"/>
+      <c r="K14" s="28" t="n"/>
+      <c r="L14" s="4" t="inlineStr"/>
+      <c r="M14" s="4" t="inlineStr"/>
+      <c r="N14" s="4" t="inlineStr"/>
+      <c r="O14" s="4" t="inlineStr"/>
+      <c r="P14" s="4" t="inlineStr"/>
+      <c r="Q14" s="4" t="inlineStr"/>
+      <c r="R14" s="4" t="inlineStr"/>
+      <c r="S14" s="4" t="inlineStr"/>
+      <c r="T14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Monday</t>
+          <t>Wednesday</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr"/>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Elective2</t>
-        </is>
-      </c>
-      <c r="D15" s="11" t="n"/>
+          <t>Elective2T</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr"/>
       <c r="E15" s="4" t="inlineStr"/>
-      <c r="F15" s="29" t="inlineStr">
-        <is>
-          <t>DA263T (C403)</t>
-        </is>
-      </c>
-      <c r="G15" s="29" t="n"/>
-      <c r="H15" s="4" t="inlineStr"/>
+      <c r="F15" s="27" t="inlineStr">
+        <is>
+          <t>DA264 (C404)</t>
+        </is>
+      </c>
+      <c r="G15" s="27" t="n"/>
+      <c r="H15" s="27" t="n"/>
       <c r="I15" s="4" t="inlineStr"/>
       <c r="J15" s="4" t="inlineStr"/>
       <c r="K15" s="4" t="inlineStr"/>
       <c r="L15" s="4" t="inlineStr"/>
-      <c r="M15" s="28" t="inlineStr">
-        <is>
-          <t>DA265 (C405)</t>
-        </is>
-      </c>
-      <c r="N15" s="28" t="n"/>
+      <c r="M15" s="25" t="inlineStr">
+        <is>
+          <t>HS261 (C403)</t>
+        </is>
+      </c>
+      <c r="N15" s="25" t="n"/>
       <c r="O15" s="4" t="inlineStr"/>
       <c r="P15" s="4" t="inlineStr"/>
       <c r="Q15" s="4" t="inlineStr"/>
@@ -10853,34 +10877,34 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Tuesday</t>
+          <t>Thursday</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr"/>
-      <c r="C16" s="11" t="inlineStr">
-        <is>
-          <t>Elective2</t>
-        </is>
-      </c>
-      <c r="D16" s="11" t="n"/>
+      <c r="C16" s="29" t="inlineStr">
+        <is>
+          <t>DA263 (C403)</t>
+        </is>
+      </c>
+      <c r="D16" s="29" t="n"/>
       <c r="E16" s="4" t="inlineStr"/>
       <c r="F16" s="27" t="inlineStr">
         <is>
-          <t>DA264 (C404)</t>
+          <t>DA264 (Lab-L406)</t>
         </is>
       </c>
       <c r="G16" s="27" t="n"/>
       <c r="H16" s="27" t="n"/>
-      <c r="I16" s="28" t="inlineStr">
-        <is>
-          <t>DA265T (C405)</t>
-        </is>
-      </c>
-      <c r="J16" s="28" t="n"/>
-      <c r="K16" s="28" t="n"/>
+      <c r="I16" s="27" t="n"/>
+      <c r="J16" s="27" t="n"/>
+      <c r="K16" s="4" t="inlineStr"/>
       <c r="L16" s="4" t="inlineStr"/>
-      <c r="M16" s="4" t="inlineStr"/>
-      <c r="N16" s="4" t="inlineStr"/>
+      <c r="M16" s="25" t="inlineStr">
+        <is>
+          <t>HS261 (C403)</t>
+        </is>
+      </c>
+      <c r="N16" s="25" t="n"/>
       <c r="O16" s="4" t="inlineStr"/>
       <c r="P16" s="4" t="inlineStr"/>
       <c r="Q16" s="4" t="inlineStr"/>
@@ -10891,34 +10915,30 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Wednesday</t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr"/>
-      <c r="C17" s="11" t="inlineStr">
-        <is>
-          <t>Elective2T</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr"/>
+      <c r="C17" s="28" t="inlineStr">
+        <is>
+          <t>DA265 (C405)</t>
+        </is>
+      </c>
+      <c r="D17" s="28" t="n"/>
       <c r="E17" s="4" t="inlineStr"/>
-      <c r="F17" s="27" t="inlineStr">
-        <is>
-          <t>DA264 (C404)</t>
-        </is>
-      </c>
-      <c r="G17" s="27" t="n"/>
-      <c r="H17" s="27" t="n"/>
+      <c r="F17" s="29" t="inlineStr">
+        <is>
+          <t>DA263 (C403)</t>
+        </is>
+      </c>
+      <c r="G17" s="29" t="n"/>
+      <c r="H17" s="29" t="n"/>
       <c r="I17" s="4" t="inlineStr"/>
       <c r="J17" s="4" t="inlineStr"/>
       <c r="K17" s="4" t="inlineStr"/>
       <c r="L17" s="4" t="inlineStr"/>
-      <c r="M17" s="25" t="inlineStr">
-        <is>
-          <t>HS261 (C403)</t>
-        </is>
-      </c>
-      <c r="N17" s="25" t="n"/>
+      <c r="M17" s="4" t="inlineStr"/>
+      <c r="N17" s="4" t="inlineStr"/>
       <c r="O17" s="4" t="inlineStr"/>
       <c r="P17" s="4" t="inlineStr"/>
       <c r="Q17" s="4" t="inlineStr"/>
@@ -10927,83 +10947,51 @@
       <c r="T17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Thursday</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr"/>
-      <c r="C18" s="29" t="inlineStr">
-        <is>
-          <t>DA263 (C403)</t>
-        </is>
-      </c>
-      <c r="D18" s="29" t="n"/>
-      <c r="E18" s="4" t="inlineStr"/>
-      <c r="F18" s="27" t="inlineStr">
-        <is>
-          <t>DA264 (Lab-L406)</t>
-        </is>
-      </c>
-      <c r="G18" s="27" t="n"/>
-      <c r="H18" s="27" t="n"/>
-      <c r="I18" s="27" t="n"/>
-      <c r="J18" s="27" t="n"/>
-      <c r="K18" s="4" t="inlineStr"/>
-      <c r="L18" s="4" t="inlineStr"/>
-      <c r="M18" s="25" t="inlineStr">
-        <is>
-          <t>HS261 (C403)</t>
-        </is>
-      </c>
-      <c r="N18" s="25" t="n"/>
-      <c r="O18" s="4" t="inlineStr"/>
-      <c r="P18" s="4" t="inlineStr"/>
-      <c r="Q18" s="4" t="inlineStr"/>
-      <c r="R18" s="4" t="inlineStr"/>
-      <c r="S18" s="4" t="inlineStr"/>
-      <c r="T18" s="4" t="inlineStr"/>
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" s="4" t="n"/>
+      <c r="C18" s="4" t="n"/>
+      <c r="D18" s="4" t="n"/>
+      <c r="E18" s="4" t="n"/>
+      <c r="F18" s="4" t="n"/>
+      <c r="G18" s="4" t="n"/>
+      <c r="H18" s="4" t="n"/>
+      <c r="I18" s="4" t="n"/>
+      <c r="J18" s="4" t="n"/>
+      <c r="K18" s="4" t="n"/>
+      <c r="L18" s="4" t="n"/>
+      <c r="M18" s="4" t="n"/>
+      <c r="N18" s="4" t="n"/>
+      <c r="O18" s="4" t="n"/>
+      <c r="P18" s="4" t="n"/>
+      <c r="Q18" s="4" t="n"/>
+      <c r="R18" s="4" t="n"/>
+      <c r="S18" s="4" t="n"/>
+      <c r="T18" s="4" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr"/>
-      <c r="C19" s="28" t="inlineStr">
-        <is>
-          <t>DA265 (C405)</t>
-        </is>
-      </c>
-      <c r="D19" s="28" t="n"/>
-      <c r="E19" s="4" t="inlineStr"/>
-      <c r="F19" s="29" t="inlineStr">
-        <is>
-          <t>DA263 (C403)</t>
-        </is>
-      </c>
-      <c r="G19" s="29" t="n"/>
-      <c r="H19" s="29" t="n"/>
-      <c r="I19" s="4" t="inlineStr"/>
-      <c r="J19" s="4" t="inlineStr"/>
-      <c r="K19" s="4" t="inlineStr"/>
-      <c r="L19" s="4" t="inlineStr"/>
-      <c r="M19" s="4" t="inlineStr"/>
-      <c r="N19" s="4" t="inlineStr"/>
-      <c r="O19" s="4" t="inlineStr"/>
-      <c r="P19" s="4" t="inlineStr"/>
-      <c r="Q19" s="4" t="inlineStr"/>
-      <c r="R19" s="4" t="inlineStr"/>
-      <c r="S19" s="4" t="inlineStr"/>
-      <c r="T19" s="4" t="inlineStr"/>
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" s="4" t="n"/>
+      <c r="C19" s="4" t="n"/>
+      <c r="D19" s="4" t="n"/>
+      <c r="E19" s="4" t="n"/>
+      <c r="F19" s="4" t="n"/>
+      <c r="G19" s="4" t="n"/>
+      <c r="H19" s="4" t="n"/>
+      <c r="I19" s="4" t="n"/>
+      <c r="J19" s="4" t="n"/>
+      <c r="K19" s="4" t="n"/>
+      <c r="L19" s="4" t="n"/>
+      <c r="M19" s="4" t="n"/>
+      <c r="N19" s="4" t="n"/>
+      <c r="O19" s="4" t="n"/>
+      <c r="P19" s="4" t="n"/>
+      <c r="Q19" s="4" t="n"/>
+      <c r="R19" s="4" t="n"/>
+      <c r="S19" s="4" t="n"/>
+      <c r="T19" s="4" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>WARNING: Courses missing from generated timetable output</t>
-        </is>
-      </c>
+      <c r="A20" t="inlineStr"/>
       <c r="B20" s="4" t="n"/>
       <c r="C20" s="4" t="n"/>
       <c r="D20" s="4" t="n"/>
@@ -11025,9 +11013,9 @@
       <c r="T20" s="4" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>DS308: combined-course constraints prevented placement</t>
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>Legend - DSAI IV</t>
         </is>
       </c>
       <c r="B21" s="4" t="n"/>
@@ -11051,14 +11039,46 @@
       <c r="T21" s="4" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
-      <c r="B22" s="4" t="n"/>
-      <c r="C22" s="4" t="n"/>
-      <c r="D22" s="4" t="n"/>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="4" t="n"/>
-      <c r="G22" s="4" t="n"/>
-      <c r="H22" s="4" t="n"/>
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>Course Code</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>Course Title</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>L-T-P-S-C</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>Faculty</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="inlineStr">
+        <is>
+          <t>Semester Half</t>
+        </is>
+      </c>
+      <c r="F22" s="16" t="inlineStr">
+        <is>
+          <t>Elective</t>
+        </is>
+      </c>
+      <c r="G22" s="16" t="inlineStr">
+        <is>
+          <t>Elective Basket</t>
+        </is>
+      </c>
+      <c r="H22" s="16" t="inlineStr">
+        <is>
+          <t>Elective Room</t>
+        </is>
+      </c>
       <c r="I22" s="4" t="n"/>
       <c r="J22" s="4" t="n"/>
       <c r="K22" s="4" t="n"/>
@@ -11073,14 +11093,42 @@
       <c r="T22" s="4" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
-      <c r="B23" s="4" t="n"/>
-      <c r="C23" s="4" t="n"/>
-      <c r="D23" s="4" t="n"/>
-      <c r="E23" s="4" t="n"/>
-      <c r="F23" s="4" t="n"/>
-      <c r="G23" s="4" t="n"/>
-      <c r="H23" s="4" t="n"/>
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>DA263</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Big Data Analytics</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>3-1-0-0-4</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Animesh Chaturvedi</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Full Sem</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr"/>
       <c r="I23" s="4" t="n"/>
       <c r="J23" s="4" t="n"/>
       <c r="K23" s="4" t="n"/>
@@ -11095,14 +11143,42 @@
       <c r="T23" s="4" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr"/>
-      <c r="B24" s="4" t="n"/>
-      <c r="C24" s="4" t="n"/>
-      <c r="D24" s="4" t="n"/>
-      <c r="E24" s="4" t="n"/>
-      <c r="F24" s="4" t="n"/>
-      <c r="G24" s="4" t="n"/>
-      <c r="H24" s="4" t="n"/>
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>DA264</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Database Management and Warehousing</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>3-0-2-0-4</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Utkarsh Mahadeo Khaire</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Full Sem</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr"/>
       <c r="I24" s="4" t="n"/>
       <c r="J24" s="4" t="n"/>
       <c r="K24" s="4" t="n"/>
@@ -11117,18 +11193,42 @@
       <c r="T24" s="4" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="inlineStr">
-        <is>
-          <t>Legend - DSAI IV</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="n"/>
-      <c r="C25" s="4" t="n"/>
-      <c r="D25" s="4" t="n"/>
-      <c r="E25" s="4" t="n"/>
-      <c r="F25" s="4" t="n"/>
-      <c r="G25" s="4" t="n"/>
-      <c r="H25" s="4" t="n"/>
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>DA265</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Deep Learning</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>3-1-0-0-4</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Shirshendu Layek</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Full Sem</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr"/>
       <c r="I25" s="4" t="n"/>
       <c r="J25" s="4" t="n"/>
       <c r="K25" s="4" t="n"/>
@@ -11143,46 +11243,42 @@
       <c r="T25" s="4" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="14" t="inlineStr">
-        <is>
-          <t>Course Code</t>
-        </is>
-      </c>
-      <c r="B26" s="15" t="inlineStr">
-        <is>
-          <t>Course Title</t>
-        </is>
-      </c>
-      <c r="C26" s="15" t="inlineStr">
-        <is>
-          <t>L-T-P-S-C</t>
-        </is>
-      </c>
-      <c r="D26" s="15" t="inlineStr">
-        <is>
-          <t>Faculty</t>
-        </is>
-      </c>
-      <c r="E26" s="15" t="inlineStr">
-        <is>
-          <t>Semester Half</t>
-        </is>
-      </c>
-      <c r="F26" s="16" t="inlineStr">
-        <is>
-          <t>Elective</t>
-        </is>
-      </c>
-      <c r="G26" s="16" t="inlineStr">
-        <is>
-          <t>Elective Basket</t>
-        </is>
-      </c>
-      <c r="H26" s="16" t="inlineStr">
-        <is>
-          <t>Elective Room</t>
-        </is>
-      </c>
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>DS308</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Data Security and Privacy</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>3-1-0-4-4</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Girish Revadigar</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Full Sem</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr"/>
       <c r="I26" s="4" t="n"/>
       <c r="J26" s="4" t="n"/>
       <c r="K26" s="4" t="n"/>
@@ -11199,22 +11295,22 @@
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
         <is>
-          <t>DA263</t>
+          <t>HS261</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Big Data Analytics</t>
+          <t>Ethics and Values / Environmental Studies</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>3-1-0-0-4</t>
+          <t>3-0-0-0-3</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Dr. Animesh Chaturvedi</t>
+          <t>Dr. Aswath Babu H</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -11249,40 +11345,44 @@
     <row r="28">
       <c r="A28" s="17" t="inlineStr">
         <is>
-          <t>DA264</t>
+          <t>EC255</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Database Management and Warehousing</t>
+          <t>Embedded Intelligent Sensing Systems</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>3-0-2-0-4</t>
+          <t>2-0-2-4-2</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Dr. Utkarsh Mahadeo Khaire</t>
+          <t>Dr. Sibasankar Padhy</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Full Sem</t>
+          <t>First Half</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>C301</t>
+        </is>
+      </c>
       <c r="I28" s="4" t="n"/>
       <c r="J28" s="4" t="n"/>
       <c r="K28" s="4" t="n"/>
@@ -11299,40 +11399,44 @@
     <row r="29">
       <c r="A29" s="17" t="inlineStr">
         <is>
-          <t>DA265</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Deep Learning</t>
+          <t>Edge AI Systems Design</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>3-1-0-0-4</t>
+          <t>3-1-0-0-2</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Dr. Shirshendu Layek</t>
+          <t>Dr. Deepak K T</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Full Sem</t>
+          <t>First Half</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>C102</t>
+        </is>
+      </c>
       <c r="I29" s="4" t="n"/>
       <c r="J29" s="4" t="n"/>
       <c r="K29" s="4" t="n"/>
@@ -11349,40 +11453,44 @@
     <row r="30">
       <c r="A30" s="17" t="inlineStr">
         <is>
-          <t>DS308</t>
+          <t>CS252</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Data Security and Privacy</t>
+          <t>Digital Forensic</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>3-1-0-4-4</t>
+          <t>3-1-0-0-2</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Dr. Girish Revadigar</t>
+          <t>Dr. Abdul Wahid</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Full Sem</t>
+          <t>Second Half</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H30" s="4" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>C401</t>
+        </is>
+      </c>
       <c r="I30" s="4" t="n"/>
       <c r="J30" s="4" t="n"/>
       <c r="K30" s="4" t="n"/>
@@ -11399,40 +11507,44 @@
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>HS261</t>
+          <t>CS261</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Ethics and Values / Environmental Studies</t>
+          <t>Operating System</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>3-0-0-0-3</t>
+          <t>3-1-0-0-2</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Dr. Aswath Babu H</t>
+          <t>Dr. Siddharth R</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Full Sem</t>
+          <t>Second Half</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H31" s="4" t="inlineStr"/>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>C003</t>
+        </is>
+      </c>
       <c r="I31" s="4" t="n"/>
       <c r="J31" s="4" t="n"/>
       <c r="K31" s="4" t="n"/>
@@ -11449,27 +11561,27 @@
     <row r="32">
       <c r="A32" s="17" t="inlineStr">
         <is>
-          <t>EC255</t>
+          <t>EC257</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Embedded Intelligent Sensing Systems</t>
+          <t>Causal Inference</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>2-0-2-4-2</t>
+          <t>3-1-0-0-2</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Dr. Sibasankar Padhy</t>
+          <t>Dr. Chinmayananda A</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>First Half</t>
+          <t>Second Half</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
@@ -11479,12 +11591,12 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>C301</t>
+          <t>C302</t>
         </is>
       </c>
       <c r="I32" s="4" t="n"/>
@@ -11503,12 +11615,12 @@
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>CS253</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Edge AI Systems Design</t>
+          <t>Time Series Forecasting and Applications</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -11518,12 +11630,12 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Dr. Deepak K T</t>
+          <t>Dr. Nataraj</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>First Half</t>
+          <t>Second Half</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
@@ -11533,12 +11645,12 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>C102</t>
+          <t>C303</t>
         </is>
       </c>
       <c r="I33" s="4" t="n"/>
@@ -11555,46 +11667,14 @@
       <c r="T33" s="4" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="17" t="inlineStr">
-        <is>
-          <t>CS252</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>Digital Forensic</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>3-1-0-0-2</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>Dr. Abdul Wahid</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>Second Half</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>C401</t>
-        </is>
-      </c>
+      <c r="A34" t="inlineStr"/>
+      <c r="B34" s="4" t="n"/>
+      <c r="C34" s="4" t="n"/>
+      <c r="D34" s="4" t="n"/>
+      <c r="E34" s="4" t="n"/>
+      <c r="F34" s="4" t="n"/>
+      <c r="G34" s="4" t="n"/>
+      <c r="H34" s="4" t="n"/>
       <c r="I34" s="4" t="n"/>
       <c r="J34" s="4" t="n"/>
       <c r="K34" s="4" t="n"/>
@@ -11608,216 +11688,32 @@
       <c r="S34" s="4" t="n"/>
       <c r="T34" s="4" t="n"/>
     </row>
-    <row r="35">
-      <c r="A35" s="17" t="inlineStr">
-        <is>
-          <t>CS261</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>Operating System</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>3-1-0-0-2</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>Dr. Siddharth R</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>Second Half</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H35" s="3" t="inlineStr">
-        <is>
-          <t>C003</t>
-        </is>
-      </c>
-      <c r="I35" s="4" t="n"/>
-      <c r="J35" s="4" t="n"/>
-      <c r="K35" s="4" t="n"/>
-      <c r="L35" s="4" t="n"/>
-      <c r="M35" s="4" t="n"/>
-      <c r="N35" s="4" t="n"/>
-      <c r="O35" s="4" t="n"/>
-      <c r="P35" s="4" t="n"/>
-      <c r="Q35" s="4" t="n"/>
-      <c r="R35" s="4" t="n"/>
-      <c r="S35" s="4" t="n"/>
-      <c r="T35" s="4" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="17" t="inlineStr">
-        <is>
-          <t>EC257</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>Causal Inference</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>3-1-0-0-2</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>Dr. Chinmayananda A</t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="inlineStr">
-        <is>
-          <t>Second Half</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G36" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H36" s="3" t="inlineStr">
-        <is>
-          <t>C302</t>
-        </is>
-      </c>
-      <c r="I36" s="4" t="n"/>
-      <c r="J36" s="4" t="n"/>
-      <c r="K36" s="4" t="n"/>
-      <c r="L36" s="4" t="n"/>
-      <c r="M36" s="4" t="n"/>
-      <c r="N36" s="4" t="n"/>
-      <c r="O36" s="4" t="n"/>
-      <c r="P36" s="4" t="n"/>
-      <c r="Q36" s="4" t="n"/>
-      <c r="R36" s="4" t="n"/>
-      <c r="S36" s="4" t="n"/>
-      <c r="T36" s="4" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="17" t="inlineStr">
-        <is>
-          <t>CS253</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>Time Series Forecasting and Applications</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>3-1-0-0-2</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>Dr. Nataraj</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>Second Half</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G37" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr">
-        <is>
-          <t>C303</t>
-        </is>
-      </c>
-      <c r="I37" s="4" t="n"/>
-      <c r="J37" s="4" t="n"/>
-      <c r="K37" s="4" t="n"/>
-      <c r="L37" s="4" t="n"/>
-      <c r="M37" s="4" t="n"/>
-      <c r="N37" s="4" t="n"/>
-      <c r="O37" s="4" t="n"/>
-      <c r="P37" s="4" t="n"/>
-      <c r="Q37" s="4" t="n"/>
-      <c r="R37" s="4" t="n"/>
-      <c r="S37" s="4" t="n"/>
-      <c r="T37" s="4" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr"/>
-      <c r="B38" s="4" t="n"/>
-      <c r="C38" s="4" t="n"/>
-      <c r="D38" s="4" t="n"/>
-      <c r="E38" s="4" t="n"/>
-      <c r="F38" s="4" t="n"/>
-      <c r="G38" s="4" t="n"/>
-      <c r="H38" s="4" t="n"/>
-      <c r="I38" s="4" t="n"/>
-      <c r="J38" s="4" t="n"/>
-      <c r="K38" s="4" t="n"/>
-      <c r="L38" s="4" t="n"/>
-      <c r="M38" s="4" t="n"/>
-      <c r="N38" s="4" t="n"/>
-      <c r="O38" s="4" t="n"/>
-      <c r="P38" s="4" t="n"/>
-      <c r="Q38" s="4" t="n"/>
-      <c r="R38" s="4" t="n"/>
-      <c r="S38" s="4" t="n"/>
-      <c r="T38" s="4" t="n"/>
-    </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="I16:K16"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="F5:H5"/>
-    <mergeCell ref="C15:D15"/>
     <mergeCell ref="O4:Q4"/>
+    <mergeCell ref="F16:J16"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="F8:H8"/>
+    <mergeCell ref="C14:D14"/>
     <mergeCell ref="M5:N5"/>
     <mergeCell ref="F17:H17"/>
     <mergeCell ref="F6:J6"/>
-    <mergeCell ref="C18:D18"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="C16:D16"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="F18:J18"/>
+    <mergeCell ref="I14:K14"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="M16:N16"/>
     <mergeCell ref="M15:N15"/>
+    <mergeCell ref="F14:H14"/>
     <mergeCell ref="M6:N6"/>
-    <mergeCell ref="M18:N18"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="F16:H16"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="C17:D17"/>
     <mergeCell ref="C7:D7"/>
-    <mergeCell ref="F19:H19"/>
-    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C13:D13"/>
     <mergeCell ref="F7:H7"/>
+    <mergeCell ref="F15:H15"/>
     <mergeCell ref="M4:N4"/>
     <mergeCell ref="F4:J4"/>
   </mergeCells>

</xml_diff>